<commit_message>
Integrate 4.0.4: commit #49233ba, 3/3/25, Update phaseout timeline for battery ITC
</commit_message>
<xml_diff>
--- a/InputData/elec/BPSpUGBCD/BAU Subsidy per Unit Grid Battery Capacity Deployed.xlsx
+++ b/InputData/elec/BPSpUGBCD/BAU Subsidy per Unit Grid Battery Capacity Deployed.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\elec\BPSpUGBCD\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanO'Brien\Models\EPS\US\eps-us\InputData\elec\BPSpUGBCD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AF49387-40D7-4827-B5F4-11DFF6188CAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D378A23B-1048-4F0E-9691-78F9E5763631}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1320" yWindow="1200" windowWidth="24750" windowHeight="14490" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -479,7 +479,7 @@
     <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.0"/>
     <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="18">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1346,14 +1346,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -1361,27 +1361,27 @@
         <v>60</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:2">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>7</v>
       </c>
@@ -1398,7 +1398,7 @@
     <tabColor rgb="FF6AA84F"/>
   </sheetPr>
   <dimension ref="A1:BV252"/>
-  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="94.42578125" style="6" customWidth="1"/>
     <col min="2" max="2" width="15.42578125" style="6" customWidth="1"/>
@@ -1410,7 +1410,7 @@
     <col min="37" max="16384" width="12.5703125" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:37" ht="12.75">
+    <row r="1" spans="1:37" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
         <v>8</v>
       </c>
@@ -1450,7 +1450,7 @@
       <c r="AI1" s="5"/>
       <c r="AJ1" s="5"/>
     </row>
-    <row r="2" spans="1:37" ht="305.25" customHeight="1">
+    <row r="2" spans="1:37" ht="305.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="7" t="s">
         <v>62</v>
       </c>
@@ -1490,7 +1490,7 @@
       <c r="AI2" s="5"/>
       <c r="AJ2" s="5"/>
     </row>
-    <row r="3" spans="1:37" ht="12.75">
+    <row r="3" spans="1:37" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A3" s="5"/>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
@@ -1528,7 +1528,7 @@
       <c r="AI3" s="5"/>
       <c r="AJ3" s="5"/>
     </row>
-    <row r="4" spans="1:37" ht="12.75">
+    <row r="4" spans="1:37" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
         <v>63</v>
       </c>
@@ -1568,7 +1568,7 @@
       <c r="AI4" s="5"/>
       <c r="AJ4" s="5"/>
     </row>
-    <row r="5" spans="1:37" ht="12.75">
+    <row r="5" spans="1:37" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
         <v>64</v>
       </c>
@@ -1608,7 +1608,7 @@
       <c r="AI5" s="5"/>
       <c r="AJ5" s="5"/>
     </row>
-    <row r="6" spans="1:37" ht="12.75">
+    <row r="6" spans="1:37" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
         <v>65</v>
       </c>
@@ -1648,7 +1648,7 @@
       <c r="AI6" s="5"/>
       <c r="AJ6" s="5"/>
     </row>
-    <row r="7" spans="1:37" ht="12.75">
+    <row r="7" spans="1:37" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
         <v>66</v>
       </c>
@@ -1688,7 +1688,7 @@
       <c r="AI7" s="5"/>
       <c r="AJ7" s="5"/>
     </row>
-    <row r="8" spans="1:37" ht="12.75">
+    <row r="8" spans="1:37" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A8" s="5">
         <f>1554.4*0.25</f>
         <v>388.6</v>
@@ -1731,7 +1731,7 @@
       <c r="AI8" s="5"/>
       <c r="AJ8" s="5"/>
     </row>
-    <row r="9" spans="1:37" ht="12.75">
+    <row r="9" spans="1:37" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
         <v>130</v>
       </c>
@@ -1771,7 +1771,7 @@
       <c r="AI9" s="5"/>
       <c r="AJ9" s="5"/>
     </row>
-    <row r="10" spans="1:37" ht="12.75">
+    <row r="10" spans="1:37" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
         <v>68</v>
       </c>
@@ -1811,7 +1811,7 @@
       <c r="AI10" s="5"/>
       <c r="AJ10" s="5"/>
     </row>
-    <row r="11" spans="1:37" ht="12.75">
+    <row r="11" spans="1:37" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A11" s="5"/>
       <c r="B11" s="5"/>
       <c r="C11" s="5"/>
@@ -1849,7 +1849,7 @@
       <c r="AI11" s="5"/>
       <c r="AJ11" s="5"/>
     </row>
-    <row r="12" spans="1:37" ht="12.75">
+    <row r="12" spans="1:37" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
         <v>69</v>
       </c>
@@ -1895,7 +1895,7 @@
       <c r="AI12" s="5"/>
       <c r="AJ12" s="5"/>
     </row>
-    <row r="13" spans="1:37" ht="12.75">
+    <row r="13" spans="1:37" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A13" s="41">
         <v>1</v>
       </c>
@@ -1941,7 +1941,7 @@
       <c r="AI13" s="5"/>
       <c r="AJ13" s="5"/>
     </row>
-    <row r="14" spans="1:37" ht="12.75">
+    <row r="14" spans="1:37" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A14" s="41"/>
       <c r="B14" s="41"/>
       <c r="C14" s="41"/>
@@ -1987,7 +1987,7 @@
       <c r="AI14" s="5"/>
       <c r="AJ14" s="5"/>
     </row>
-    <row r="15" spans="1:37" ht="12.75">
+    <row r="15" spans="1:37" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A15" s="41" t="s">
         <v>77</v>
       </c>
@@ -2027,7 +2027,7 @@
       <c r="AI15" s="5"/>
       <c r="AJ15" s="5"/>
     </row>
-    <row r="16" spans="1:37" ht="12.75">
+    <row r="16" spans="1:37" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A16" s="6">
         <v>2020</v>
       </c>
@@ -2128,7 +2128,7 @@
       <c r="AJ16" s="42"/>
       <c r="AK16" s="42"/>
     </row>
-    <row r="17" spans="1:51" ht="12.75">
+    <row r="17" spans="1:51" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A17" s="41">
         <v>1</v>
       </c>
@@ -2181,13 +2181,13 @@
         <v>1</v>
       </c>
       <c r="R17" s="41">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="S17" s="41">
-        <v>0.75</v>
+        <v>0.5</v>
       </c>
       <c r="T17" s="41">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="U17" s="41">
         <v>0</v>
@@ -2243,7 +2243,7 @@
       <c r="AX17" s="41"/>
       <c r="AY17" s="41"/>
     </row>
-    <row r="18" spans="1:51" ht="12.75">
+    <row r="18" spans="1:51" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A18" s="5"/>
       <c r="B18" s="5"/>
       <c r="C18" s="5"/>
@@ -2281,7 +2281,7 @@
       <c r="AI18" s="5"/>
       <c r="AJ18" s="5"/>
     </row>
-    <row r="19" spans="1:51" ht="12.75">
+    <row r="19" spans="1:51" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A19" s="4" t="s">
         <v>9</v>
       </c>
@@ -2321,7 +2321,7 @@
       <c r="AI19" s="8"/>
       <c r="AJ19" s="8"/>
     </row>
-    <row r="20" spans="1:51" ht="12.75">
+    <row r="20" spans="1:51" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A20" s="9" t="s">
         <v>10</v>
       </c>
@@ -2361,7 +2361,7 @@
       <c r="AI20" s="10"/>
       <c r="AJ20" s="10"/>
     </row>
-    <row r="21" spans="1:51" ht="12.75">
+    <row r="21" spans="1:51" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A21" s="11" t="s">
         <v>11</v>
       </c>
@@ -2401,7 +2401,7 @@
       <c r="AI21" s="5"/>
       <c r="AJ21" s="5"/>
     </row>
-    <row r="22" spans="1:51" ht="12.75">
+    <row r="22" spans="1:51" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A22" s="12" t="s">
         <v>12</v>
       </c>
@@ -2441,7 +2441,7 @@
       <c r="AI22" s="5"/>
       <c r="AJ22" s="5"/>
     </row>
-    <row r="23" spans="1:51" ht="12.75">
+    <row r="23" spans="1:51" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A23" s="13"/>
       <c r="B23" s="5"/>
       <c r="C23" s="5"/>
@@ -2479,7 +2479,7 @@
       <c r="AI23" s="5"/>
       <c r="AJ23" s="5"/>
     </row>
-    <row r="24" spans="1:51" ht="12.75">
+    <row r="24" spans="1:51" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A24" s="13"/>
       <c r="B24" s="5"/>
       <c r="C24" s="5"/>
@@ -2517,7 +2517,7 @@
       <c r="AI24" s="5"/>
       <c r="AJ24" s="5"/>
     </row>
-    <row r="25" spans="1:51" ht="12.75">
+    <row r="25" spans="1:51" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A25" s="13"/>
       <c r="B25" s="5"/>
       <c r="C25" s="5"/>
@@ -2555,7 +2555,7 @@
       <c r="AI25" s="5"/>
       <c r="AJ25" s="5"/>
     </row>
-    <row r="26" spans="1:51" ht="12.75">
+    <row r="26" spans="1:51" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A26" s="13"/>
       <c r="B26" s="5"/>
       <c r="C26" s="5"/>
@@ -2593,7 +2593,7 @@
       <c r="AI26" s="5"/>
       <c r="AJ26" s="5"/>
     </row>
-    <row r="27" spans="1:51" ht="12.75">
+    <row r="27" spans="1:51" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A27" s="13"/>
       <c r="B27" s="5"/>
       <c r="C27" s="5"/>
@@ -2631,7 +2631,7 @@
       <c r="AI27" s="5"/>
       <c r="AJ27" s="5"/>
     </row>
-    <row r="28" spans="1:51" ht="12.75">
+    <row r="28" spans="1:51" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A28" s="13"/>
       <c r="B28" s="5"/>
       <c r="C28" s="5"/>
@@ -2669,7 +2669,7 @@
       <c r="AI28" s="5"/>
       <c r="AJ28" s="5"/>
     </row>
-    <row r="29" spans="1:51" ht="12.75">
+    <row r="29" spans="1:51" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A29" s="13"/>
       <c r="B29" s="5"/>
       <c r="C29" s="5"/>
@@ -2707,7 +2707,7 @@
       <c r="AI29" s="5"/>
       <c r="AJ29" s="5"/>
     </row>
-    <row r="30" spans="1:51" ht="12.75">
+    <row r="30" spans="1:51" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A30" s="13"/>
       <c r="B30" s="5"/>
       <c r="C30" s="5"/>
@@ -2745,7 +2745,7 @@
       <c r="AI30" s="5"/>
       <c r="AJ30" s="5"/>
     </row>
-    <row r="31" spans="1:51" ht="12.75">
+    <row r="31" spans="1:51" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A31" s="13"/>
       <c r="B31" s="5"/>
       <c r="C31" s="5"/>
@@ -2783,7 +2783,7 @@
       <c r="AI31" s="5"/>
       <c r="AJ31" s="5"/>
     </row>
-    <row r="32" spans="1:51" ht="12.75">
+    <row r="32" spans="1:51" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A32" s="13"/>
       <c r="B32" s="5"/>
       <c r="C32" s="5"/>
@@ -2821,7 +2821,7 @@
       <c r="AI32" s="5"/>
       <c r="AJ32" s="5"/>
     </row>
-    <row r="33" spans="1:36" ht="12.75">
+    <row r="33" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A33" s="13"/>
       <c r="B33" s="5"/>
       <c r="C33" s="5"/>
@@ -2859,7 +2859,7 @@
       <c r="AI33" s="5"/>
       <c r="AJ33" s="5"/>
     </row>
-    <row r="34" spans="1:36" ht="12.75">
+    <row r="34" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A34" s="13"/>
       <c r="B34" s="5"/>
       <c r="C34" s="5"/>
@@ -2897,7 +2897,7 @@
       <c r="AI34" s="5"/>
       <c r="AJ34" s="5"/>
     </row>
-    <row r="35" spans="1:36" ht="12.75">
+    <row r="35" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A35" s="13"/>
       <c r="B35" s="5"/>
       <c r="C35" s="5"/>
@@ -2935,7 +2935,7 @@
       <c r="AI35" s="5"/>
       <c r="AJ35" s="5"/>
     </row>
-    <row r="36" spans="1:36" ht="12.75">
+    <row r="36" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A36" s="13"/>
       <c r="B36" s="5"/>
       <c r="C36" s="5"/>
@@ -2973,7 +2973,7 @@
       <c r="AI36" s="5"/>
       <c r="AJ36" s="5"/>
     </row>
-    <row r="37" spans="1:36" ht="12.75">
+    <row r="37" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A37" s="13"/>
       <c r="B37" s="5"/>
       <c r="C37" s="5"/>
@@ -3011,7 +3011,7 @@
       <c r="AI37" s="5"/>
       <c r="AJ37" s="5"/>
     </row>
-    <row r="38" spans="1:36" ht="12.75">
+    <row r="38" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A38" s="13"/>
       <c r="B38" s="5"/>
       <c r="C38" s="5"/>
@@ -3049,7 +3049,7 @@
       <c r="AI38" s="5"/>
       <c r="AJ38" s="5"/>
     </row>
-    <row r="39" spans="1:36" ht="12.75">
+    <row r="39" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A39" s="13"/>
       <c r="B39" s="5"/>
       <c r="C39" s="5"/>
@@ -3087,7 +3087,7 @@
       <c r="AI39" s="5"/>
       <c r="AJ39" s="5"/>
     </row>
-    <row r="40" spans="1:36" ht="12.75">
+    <row r="40" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A40" s="13"/>
       <c r="B40" s="5"/>
       <c r="C40" s="5"/>
@@ -3125,7 +3125,7 @@
       <c r="AI40" s="5"/>
       <c r="AJ40" s="5"/>
     </row>
-    <row r="41" spans="1:36" ht="12.75">
+    <row r="41" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A41" s="5" t="s">
         <v>13</v>
       </c>
@@ -3165,7 +3165,7 @@
       <c r="AI41" s="5"/>
       <c r="AJ41" s="5"/>
     </row>
-    <row r="42" spans="1:36" ht="12.75">
+    <row r="42" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A42" s="5" t="s">
         <v>14</v>
       </c>
@@ -3205,7 +3205,7 @@
       <c r="AI42" s="5"/>
       <c r="AJ42" s="5"/>
     </row>
-    <row r="43" spans="1:36" ht="12.75">
+    <row r="43" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A43" s="5" t="s">
         <v>15</v>
       </c>
@@ -3245,7 +3245,7 @@
       <c r="AI43" s="5"/>
       <c r="AJ43" s="5"/>
     </row>
-    <row r="44" spans="1:36" ht="12.75">
+    <row r="44" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A44" s="5" t="s">
         <v>78</v>
       </c>
@@ -3285,7 +3285,7 @@
       <c r="AI44" s="5"/>
       <c r="AJ44" s="5"/>
     </row>
-    <row r="45" spans="1:36" ht="12.75">
+    <row r="45" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A45" s="6" t="s">
         <v>16</v>
       </c>
@@ -3327,7 +3327,7 @@
       <c r="AI45" s="5"/>
       <c r="AJ45" s="5"/>
     </row>
-    <row r="46" spans="1:36" ht="12.75">
+    <row r="46" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A46" s="6" t="s">
         <v>17</v>
       </c>
@@ -3370,7 +3370,7 @@
       <c r="AI46" s="5"/>
       <c r="AJ46" s="5"/>
     </row>
-    <row r="47" spans="1:36" ht="12.75">
+    <row r="47" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A47" s="13"/>
       <c r="B47" s="5"/>
       <c r="C47" s="5"/>
@@ -3408,7 +3408,7 @@
       <c r="AI47" s="5"/>
       <c r="AJ47" s="5"/>
     </row>
-    <row r="48" spans="1:36" ht="12.75">
+    <row r="48" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A48" s="13"/>
       <c r="B48" s="13">
         <v>2022</v>
@@ -3504,7 +3504,7 @@
       <c r="AI48" s="5"/>
       <c r="AJ48" s="5"/>
     </row>
-    <row r="49" spans="1:36" ht="12.75">
+    <row r="49" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A49" s="15" t="s">
         <v>18</v>
       </c>
@@ -3602,7 +3602,7 @@
       <c r="AI49" s="5"/>
       <c r="AJ49" s="5"/>
     </row>
-    <row r="50" spans="1:36" ht="12.75">
+    <row r="50" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A50" s="15" t="s">
         <v>19</v>
       </c>
@@ -3701,7 +3701,7 @@
       <c r="AI50" s="5"/>
       <c r="AJ50" s="5"/>
     </row>
-    <row r="51" spans="1:36" ht="12.75">
+    <row r="51" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A51" s="13"/>
       <c r="B51" s="5"/>
       <c r="C51" s="5"/>
@@ -3739,7 +3739,7 @@
       <c r="AI51" s="5"/>
       <c r="AJ51" s="5"/>
     </row>
-    <row r="52" spans="1:36" ht="12.75">
+    <row r="52" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A52" s="9" t="s">
         <v>20</v>
       </c>
@@ -3779,7 +3779,7 @@
       <c r="AI52" s="10"/>
       <c r="AJ52" s="10"/>
     </row>
-    <row r="53" spans="1:36" ht="12.75">
+    <row r="53" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A53" s="5" t="s">
         <v>21</v>
       </c>
@@ -3819,7 +3819,7 @@
       <c r="AI53" s="5"/>
       <c r="AJ53" s="5"/>
     </row>
-    <row r="54" spans="1:36" ht="12.75">
+    <row r="54" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A54" s="16" t="s">
         <v>22</v>
       </c>
@@ -3859,7 +3859,7 @@
       <c r="AI54" s="5"/>
       <c r="AJ54" s="5"/>
     </row>
-    <row r="55" spans="1:36" ht="12.75">
+    <row r="55" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A55" s="13"/>
       <c r="B55" s="5"/>
       <c r="C55" s="5"/>
@@ -3897,7 +3897,7 @@
       <c r="AI55" s="5"/>
       <c r="AJ55" s="5"/>
     </row>
-    <row r="56" spans="1:36" ht="12.75">
+    <row r="56" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A56" s="17" t="s">
         <v>23</v>
       </c>
@@ -3941,7 +3941,7 @@
       <c r="AI56" s="5"/>
       <c r="AJ56" s="5"/>
     </row>
-    <row r="57" spans="1:36" ht="12.75">
+    <row r="57" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A57" s="19" t="s">
         <v>26</v>
       </c>
@@ -3983,7 +3983,7 @@
       <c r="AI57" s="5"/>
       <c r="AJ57" s="5"/>
     </row>
-    <row r="58" spans="1:36" ht="12.75">
+    <row r="58" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A58" s="21" t="s">
         <v>28</v>
       </c>
@@ -4027,7 +4027,7 @@
       <c r="AI58" s="5"/>
       <c r="AJ58" s="5"/>
     </row>
-    <row r="59" spans="1:36" ht="12.75">
+    <row r="59" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A59" s="21" t="s">
         <v>29</v>
       </c>
@@ -4071,7 +4071,7 @@
       <c r="AI59" s="5"/>
       <c r="AJ59" s="5"/>
     </row>
-    <row r="60" spans="1:36" ht="12.75">
+    <row r="60" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A60" s="21" t="s">
         <v>30</v>
       </c>
@@ -4115,7 +4115,7 @@
       <c r="AI60" s="5"/>
       <c r="AJ60" s="5"/>
     </row>
-    <row r="61" spans="1:36" ht="12.75">
+    <row r="61" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A61" s="21" t="s">
         <v>31</v>
       </c>
@@ -4157,7 +4157,7 @@
       <c r="AI61" s="5"/>
       <c r="AJ61" s="5"/>
     </row>
-    <row r="62" spans="1:36" ht="12.75">
+    <row r="62" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A62" s="21" t="s">
         <v>32</v>
       </c>
@@ -4199,7 +4199,7 @@
       <c r="AI62" s="5"/>
       <c r="AJ62" s="5"/>
     </row>
-    <row r="63" spans="1:36" ht="12.75">
+    <row r="63" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A63" s="21" t="s">
         <v>33</v>
       </c>
@@ -4241,7 +4241,7 @@
       <c r="AI63" s="5"/>
       <c r="AJ63" s="5"/>
     </row>
-    <row r="64" spans="1:36" ht="12.75">
+    <row r="64" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A64" s="21" t="s">
         <v>34</v>
       </c>
@@ -4283,7 +4283,7 @@
       <c r="AI64" s="5"/>
       <c r="AJ64" s="5"/>
     </row>
-    <row r="65" spans="1:36" ht="12.75">
+    <row r="65" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A65" s="21" t="s">
         <v>35</v>
       </c>
@@ -4325,7 +4325,7 @@
       <c r="AI65" s="5"/>
       <c r="AJ65" s="5"/>
     </row>
-    <row r="66" spans="1:36" ht="12.75">
+    <row r="66" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A66" s="21" t="s">
         <v>36</v>
       </c>
@@ -4367,7 +4367,7 @@
       <c r="AI66" s="5"/>
       <c r="AJ66" s="5"/>
     </row>
-    <row r="67" spans="1:36" ht="12.75">
+    <row r="67" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A67" s="24" t="s">
         <v>37</v>
       </c>
@@ -4409,7 +4409,7 @@
       <c r="AI67" s="5"/>
       <c r="AJ67" s="5"/>
     </row>
-    <row r="68" spans="1:36" ht="12.75">
+    <row r="68" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A68" s="13"/>
       <c r="B68" s="5"/>
       <c r="C68" s="5"/>
@@ -4447,7 +4447,7 @@
       <c r="AI68" s="5"/>
       <c r="AJ68" s="5"/>
     </row>
-    <row r="69" spans="1:36" ht="12.75">
+    <row r="69" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A69" s="5" t="s">
         <v>38</v>
       </c>
@@ -4490,7 +4490,7 @@
       <c r="AI69" s="5"/>
       <c r="AJ69" s="5"/>
     </row>
-    <row r="70" spans="1:36" ht="12.75">
+    <row r="70" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A70" s="5" t="s">
         <v>39</v>
       </c>
@@ -4533,7 +4533,7 @@
       <c r="AI70" s="5"/>
       <c r="AJ70" s="5"/>
     </row>
-    <row r="71" spans="1:36" ht="12.75">
+    <row r="71" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A71" s="5"/>
       <c r="B71" s="23"/>
       <c r="C71" s="5"/>
@@ -4571,7 +4571,7 @@
       <c r="AI71" s="5"/>
       <c r="AJ71" s="5"/>
     </row>
-    <row r="72" spans="1:36" ht="12.75">
+    <row r="72" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A72" s="5"/>
       <c r="B72" s="13">
         <v>2022</v>
@@ -4623,7 +4623,7 @@
       <c r="AI72" s="5"/>
       <c r="AJ72" s="5"/>
     </row>
-    <row r="73" spans="1:36" ht="12.75">
+    <row r="73" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A73" s="7" t="s">
         <v>40</v>
       </c>
@@ -4684,7 +4684,7 @@
       <c r="AI73" s="5"/>
       <c r="AJ73" s="5"/>
     </row>
-    <row r="74" spans="1:36" ht="12.75">
+    <row r="74" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A74" s="7"/>
       <c r="B74" s="7"/>
       <c r="C74" s="7"/>
@@ -4722,7 +4722,7 @@
       <c r="AI74" s="5"/>
       <c r="AJ74" s="5"/>
     </row>
-    <row r="75" spans="1:36" ht="25.5">
+    <row r="75" spans="1:36" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A75" s="7" t="s">
         <v>41</v>
       </c>
@@ -4762,7 +4762,7 @@
       <c r="AI75" s="5"/>
       <c r="AJ75" s="5"/>
     </row>
-    <row r="76" spans="1:36" ht="12.75">
+    <row r="76" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A76" s="7"/>
       <c r="B76" s="7"/>
       <c r="C76" s="7"/>
@@ -4800,7 +4800,7 @@
       <c r="AI76" s="13"/>
       <c r="AJ76" s="13"/>
     </row>
-    <row r="77" spans="1:36" s="26" customFormat="1" ht="12.75">
+    <row r="77" spans="1:36" s="26" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A77" s="15"/>
       <c r="B77" s="15">
         <v>2022</v>
@@ -4896,7 +4896,7 @@
       <c r="AI77" s="13"/>
       <c r="AJ77" s="13"/>
     </row>
-    <row r="78" spans="1:36" ht="12.75">
+    <row r="78" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A78" s="23" t="s">
         <v>42</v>
       </c>
@@ -4994,7 +4994,7 @@
       <c r="AI78" s="23"/>
       <c r="AJ78" s="23"/>
     </row>
-    <row r="79" spans="1:36" ht="12.75">
+    <row r="79" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A79" s="23" t="s">
         <v>43</v>
       </c>
@@ -5121,7 +5121,7 @@
       <c r="AI79" s="23"/>
       <c r="AJ79" s="23"/>
     </row>
-    <row r="80" spans="1:36" ht="12.75">
+    <row r="80" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A80" s="5" t="s">
         <v>44</v>
       </c>
@@ -5248,7 +5248,7 @@
       <c r="AI80" s="5"/>
       <c r="AJ80" s="5"/>
     </row>
-    <row r="81" spans="1:36" ht="12.75">
+    <row r="81" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A81" s="11"/>
       <c r="B81" s="27"/>
       <c r="C81" s="27"/>
@@ -5286,7 +5286,7 @@
       <c r="AI81" s="13"/>
       <c r="AJ81" s="13"/>
     </row>
-    <row r="82" spans="1:36" s="29" customFormat="1" ht="25.5">
+    <row r="82" spans="1:36" s="29" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A82" s="7" t="s">
         <v>45</v>
       </c>
@@ -5384,7 +5384,7 @@
       <c r="AI82" s="15"/>
       <c r="AJ82" s="15"/>
     </row>
-    <row r="83" spans="1:36" ht="12.75">
+    <row r="83" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A83" s="13"/>
       <c r="B83" s="13"/>
       <c r="C83" s="13"/>
@@ -5422,7 +5422,7 @@
       <c r="AI83" s="13"/>
       <c r="AJ83" s="13"/>
     </row>
-    <row r="84" spans="1:36" ht="12.75">
+    <row r="84" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A84" s="9" t="s">
         <v>1</v>
       </c>
@@ -5462,7 +5462,7 @@
       <c r="AI84" s="10"/>
       <c r="AJ84" s="10"/>
     </row>
-    <row r="85" spans="1:36" ht="12.75">
+    <row r="85" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A85" s="11" t="s">
         <v>46</v>
       </c>
@@ -5502,7 +5502,7 @@
       <c r="AI85" s="5"/>
       <c r="AJ85" s="5"/>
     </row>
-    <row r="86" spans="1:36" ht="12.75">
+    <row r="86" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A86" s="11" t="s">
         <v>47</v>
       </c>
@@ -5542,7 +5542,7 @@
       <c r="AI86" s="5"/>
       <c r="AJ86" s="5"/>
     </row>
-    <row r="87" spans="1:36" ht="12.75">
+    <row r="87" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A87" s="11" t="s">
         <v>48</v>
       </c>
@@ -5582,7 +5582,7 @@
       <c r="AI87" s="5"/>
       <c r="AJ87" s="5"/>
     </row>
-    <row r="88" spans="1:36" ht="12.75">
+    <row r="88" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A88" s="11" t="s">
         <v>79</v>
       </c>
@@ -5622,7 +5622,7 @@
       <c r="AI88" s="5"/>
       <c r="AJ88" s="5"/>
     </row>
-    <row r="89" spans="1:36" ht="12.75">
+    <row r="89" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A89" s="11" t="s">
         <v>80</v>
       </c>
@@ -5662,7 +5662,7 @@
       <c r="AI89" s="5"/>
       <c r="AJ89" s="5"/>
     </row>
-    <row r="90" spans="1:36" ht="12.75">
+    <row r="90" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A90" s="5"/>
       <c r="B90" s="5"/>
       <c r="C90" s="5"/>
@@ -5700,7 +5700,7 @@
       <c r="AI90" s="5"/>
       <c r="AJ90" s="5"/>
     </row>
-    <row r="91" spans="1:36" ht="12.75">
+    <row r="91" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A91" s="9" t="s">
         <v>81</v>
       </c>
@@ -5740,7 +5740,7 @@
       <c r="AI91" s="9"/>
       <c r="AJ91" s="9"/>
     </row>
-    <row r="92" spans="1:36" ht="12.75">
+    <row r="92" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A92" s="30"/>
       <c r="B92" s="30"/>
       <c r="C92" s="5"/>
@@ -5778,7 +5778,7 @@
       <c r="AI92" s="5"/>
       <c r="AJ92" s="5"/>
     </row>
-    <row r="93" spans="1:36" ht="12.75">
+    <row r="93" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A93" s="30" t="s">
         <v>82</v>
       </c>
@@ -5820,7 +5820,7 @@
       <c r="AI93" s="5"/>
       <c r="AJ93" s="5"/>
     </row>
-    <row r="94" spans="1:36" ht="12.75">
+    <row r="94" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A94" s="30" t="s">
         <v>83</v>
       </c>
@@ -5862,7 +5862,7 @@
       <c r="AI94" s="5"/>
       <c r="AJ94" s="5"/>
     </row>
-    <row r="95" spans="1:36" ht="12.75">
+    <row r="95" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A95" s="30" t="s">
         <v>84</v>
       </c>
@@ -5906,7 +5906,7 @@
       <c r="AI95" s="5"/>
       <c r="AJ95" s="5"/>
     </row>
-    <row r="96" spans="1:36" ht="12.75">
+    <row r="96" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A96" s="30" t="s">
         <v>86</v>
       </c>
@@ -5948,7 +5948,7 @@
       <c r="AI96" s="5"/>
       <c r="AJ96" s="5"/>
     </row>
-    <row r="97" spans="1:36" ht="17.25">
+    <row r="97" spans="1:36" ht="17.25" x14ac:dyDescent="0.4">
       <c r="A97" s="30" t="s">
         <v>87</v>
       </c>
@@ -5990,7 +5990,7 @@
       <c r="AI97" s="5"/>
       <c r="AJ97" s="5"/>
     </row>
-    <row r="98" spans="1:36" ht="17.25">
+    <row r="98" spans="1:36" ht="17.25" x14ac:dyDescent="0.4">
       <c r="A98" s="30"/>
       <c r="B98" s="46"/>
       <c r="C98" s="5"/>
@@ -6028,7 +6028,7 @@
       <c r="AI98" s="5"/>
       <c r="AJ98" s="5"/>
     </row>
-    <row r="99" spans="1:36" ht="12.75">
+    <row r="99" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A99" s="30" t="s">
         <v>88</v>
       </c>
@@ -6071,7 +6071,7 @@
       <c r="AI99" s="5"/>
       <c r="AJ99" s="5"/>
     </row>
-    <row r="100" spans="1:36" ht="12.75">
+    <row r="100" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A100" s="30" t="s">
         <v>89</v>
       </c>
@@ -6114,7 +6114,7 @@
       <c r="AI100" s="5"/>
       <c r="AJ100" s="5"/>
     </row>
-    <row r="101" spans="1:36" ht="12.75">
+    <row r="101" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A101" s="30" t="s">
         <v>49</v>
       </c>
@@ -6156,7 +6156,7 @@
       <c r="AI101" s="5"/>
       <c r="AJ101" s="5"/>
     </row>
-    <row r="102" spans="1:36" ht="17.25">
+    <row r="102" spans="1:36" ht="17.25" x14ac:dyDescent="0.4">
       <c r="A102" s="30" t="s">
         <v>50</v>
       </c>
@@ -6198,7 +6198,7 @@
       <c r="AI102" s="5"/>
       <c r="AJ102" s="5"/>
     </row>
-    <row r="103" spans="1:36" ht="12.75">
+    <row r="103" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A103" s="30" t="s">
         <v>90</v>
       </c>
@@ -6242,7 +6242,7 @@
       <c r="AI103" s="5"/>
       <c r="AJ103" s="5"/>
     </row>
-    <row r="104" spans="1:36" ht="12.75">
+    <row r="104" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A104" s="30" t="s">
         <v>51</v>
       </c>
@@ -6286,7 +6286,7 @@
       <c r="AI104" s="5"/>
       <c r="AJ104" s="5"/>
     </row>
-    <row r="105" spans="1:36" ht="12.75">
+    <row r="105" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A105" s="30" t="s">
         <v>52</v>
       </c>
@@ -6328,7 +6328,7 @@
       <c r="AI105" s="5"/>
       <c r="AJ105" s="5"/>
     </row>
-    <row r="106" spans="1:36" ht="12.75">
+    <row r="106" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A106" s="30" t="s">
         <v>53</v>
       </c>
@@ -6370,7 +6370,7 @@
       <c r="AI106" s="5"/>
       <c r="AJ106" s="5"/>
     </row>
-    <row r="107" spans="1:36" ht="12.75">
+    <row r="107" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A107" s="30"/>
       <c r="B107" s="30"/>
       <c r="C107" s="5"/>
@@ -6408,7 +6408,7 @@
       <c r="AI107" s="5"/>
       <c r="AJ107" s="5"/>
     </row>
-    <row r="108" spans="1:36" s="35" customFormat="1" ht="12.75">
+    <row r="108" spans="1:36" s="35" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A108" s="32" t="s">
         <v>93</v>
       </c>
@@ -6448,7 +6448,7 @@
       <c r="AI108" s="34"/>
       <c r="AJ108" s="34"/>
     </row>
-    <row r="109" spans="1:36" ht="12.75">
+    <row r="109" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A109" s="51"/>
       <c r="B109" s="30" t="s">
         <v>94</v>
@@ -6490,7 +6490,7 @@
       <c r="AI109" s="5"/>
       <c r="AJ109" s="5"/>
     </row>
-    <row r="110" spans="1:36" ht="12.75">
+    <row r="110" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A110" s="51" t="s">
         <v>96</v>
       </c>
@@ -6534,7 +6534,7 @@
       <c r="AI110" s="5"/>
       <c r="AJ110" s="5"/>
     </row>
-    <row r="111" spans="1:36" ht="12.75">
+    <row r="111" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A111" s="51"/>
       <c r="B111" s="30"/>
       <c r="C111" s="5"/>
@@ -6572,7 +6572,7 @@
       <c r="AI111" s="5"/>
       <c r="AJ111" s="5"/>
     </row>
-    <row r="112" spans="1:36" ht="12.75">
+    <row r="112" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A112" s="30"/>
       <c r="B112" s="30">
         <v>2023</v>
@@ -6665,7 +6665,7 @@
       <c r="AH112" s="5"/>
       <c r="AI112" s="5"/>
     </row>
-    <row r="113" spans="1:36" ht="12.75">
+    <row r="113" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A113" s="30" t="s">
         <v>97</v>
       </c>
@@ -6739,15 +6739,15 @@
       </c>
       <c r="S113" s="36">
         <f t="shared" si="4"/>
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="T113" s="36">
         <f t="shared" si="4"/>
-        <v>0.75</v>
+        <v>0.5</v>
       </c>
       <c r="U113" s="36">
         <f t="shared" si="4"/>
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="V113" s="36">
         <f t="shared" si="4"/>
@@ -6788,7 +6788,7 @@
       <c r="AH113" s="5"/>
       <c r="AI113" s="5"/>
     </row>
-    <row r="114" spans="1:36" ht="12.75">
+    <row r="114" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A114" s="30" t="s">
         <v>98</v>
       </c>
@@ -6854,15 +6854,15 @@
       </c>
       <c r="Q114" s="36">
         <f t="shared" si="5"/>
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="R114" s="36">
         <f t="shared" si="5"/>
-        <v>0.75</v>
+        <v>0.5</v>
       </c>
       <c r="S114" s="36">
         <f t="shared" si="5"/>
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="T114" s="36">
         <f t="shared" si="5"/>
@@ -6911,7 +6911,7 @@
       <c r="AH114" s="5"/>
       <c r="AI114" s="5"/>
     </row>
-    <row r="115" spans="1:36" ht="12.75">
+    <row r="115" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A115" s="30"/>
       <c r="B115" s="30"/>
       <c r="C115" s="5"/>
@@ -6949,7 +6949,7 @@
       <c r="AI115" s="5"/>
       <c r="AJ115" s="5"/>
     </row>
-    <row r="116" spans="1:36" ht="12.75">
+    <row r="116" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A116" s="30" t="s">
         <v>99</v>
       </c>
@@ -6989,7 +6989,7 @@
       <c r="AI116" s="5"/>
       <c r="AJ116" s="5"/>
     </row>
-    <row r="117" spans="1:36" ht="12.75">
+    <row r="117" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A117" s="30"/>
       <c r="B117" s="30">
         <v>2023</v>
@@ -7083,7 +7083,7 @@
       <c r="AI117" s="5"/>
       <c r="AJ117" s="5"/>
     </row>
-    <row r="118" spans="1:36" ht="12.75">
+    <row r="118" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A118" s="30" t="s">
         <v>100</v>
       </c>
@@ -7157,15 +7157,15 @@
       </c>
       <c r="S118" s="37">
         <f t="shared" si="6"/>
-        <v>23.620381171332561</v>
+        <v>17.715285878499422</v>
       </c>
       <c r="T118" s="37">
         <f t="shared" si="6"/>
-        <v>17.715285878499422</v>
+        <v>11.81019058566628</v>
       </c>
       <c r="U118" s="37">
         <f t="shared" si="6"/>
-        <v>11.81019058566628</v>
+        <v>0</v>
       </c>
       <c r="V118" s="37">
         <f t="shared" si="6"/>
@@ -7207,7 +7207,7 @@
       <c r="AI118" s="5"/>
       <c r="AJ118" s="5"/>
     </row>
-    <row r="119" spans="1:36" ht="12.75">
+    <row r="119" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A119" s="30"/>
       <c r="B119" s="37"/>
       <c r="C119" s="37"/>
@@ -7245,7 +7245,7 @@
       <c r="AI119" s="5"/>
       <c r="AJ119" s="5"/>
     </row>
-    <row r="120" spans="1:36" ht="12.75">
+    <row r="120" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A120" s="30" t="s">
         <v>101</v>
       </c>
@@ -7308,15 +7308,15 @@
       </c>
       <c r="Q120" s="37">
         <f t="shared" si="7"/>
-        <v>23.051383025144418</v>
+        <v>17.288537268858313</v>
       </c>
       <c r="R120" s="37">
         <f t="shared" si="7"/>
-        <v>17.288537268858313</v>
+        <v>11.525691512572209</v>
       </c>
       <c r="S120" s="37">
         <f t="shared" si="7"/>
-        <v>11.525691512572209</v>
+        <v>0</v>
       </c>
       <c r="T120" s="37">
         <f t="shared" si="7"/>
@@ -7366,7 +7366,7 @@
       <c r="AI120" s="5"/>
       <c r="AJ120" s="5"/>
     </row>
-    <row r="121" spans="1:36" ht="12.75">
+    <row r="121" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A121" s="30" t="s">
         <v>102</v>
       </c>
@@ -7406,7 +7406,7 @@
       <c r="AI121" s="5"/>
       <c r="AJ121" s="5"/>
     </row>
-    <row r="122" spans="1:36" ht="12.75">
+    <row r="122" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A122" s="30"/>
       <c r="B122" s="37"/>
       <c r="C122" s="37"/>
@@ -7444,7 +7444,7 @@
       <c r="AI122" s="5"/>
       <c r="AJ122" s="5"/>
     </row>
-    <row r="123" spans="1:36" ht="12.75">
+    <row r="123" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A123" s="30" t="s">
         <v>103</v>
       </c>
@@ -7550,7 +7550,7 @@
       <c r="AI123" s="5"/>
       <c r="AJ123" s="5"/>
     </row>
-    <row r="124" spans="1:36" ht="12.75">
+    <row r="124" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A124" s="30"/>
       <c r="B124" s="37"/>
       <c r="C124" s="37"/>
@@ -7588,7 +7588,7 @@
       <c r="AI124" s="5"/>
       <c r="AJ124" s="5"/>
     </row>
-    <row r="125" spans="1:36" s="35" customFormat="1" ht="12.75">
+    <row r="125" spans="1:36" s="35" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A125" s="32" t="s">
         <v>54</v>
       </c>
@@ -7628,7 +7628,7 @@
       <c r="AI125" s="34"/>
       <c r="AJ125" s="34"/>
     </row>
-    <row r="126" spans="1:36" ht="25.5">
+    <row r="126" spans="1:36" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A126" s="51"/>
       <c r="B126" s="5" t="s">
         <v>104</v>
@@ -7675,7 +7675,7 @@
       <c r="AH126" s="5"/>
       <c r="AI126" s="5"/>
     </row>
-    <row r="127" spans="1:36" ht="12.75">
+    <row r="127" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A127" s="51" t="s">
         <v>96</v>
       </c>
@@ -7724,7 +7724,7 @@
       <c r="AH127" s="5"/>
       <c r="AI127" s="5"/>
     </row>
-    <row r="128" spans="1:36" ht="12.75">
+    <row r="128" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A128" s="51"/>
       <c r="B128" s="37"/>
       <c r="C128" s="37"/>
@@ -7762,7 +7762,7 @@
       <c r="AI128" s="5"/>
       <c r="AJ128" s="5"/>
     </row>
-    <row r="129" spans="1:36" ht="12.75">
+    <row r="129" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A129" s="30" t="s">
         <v>55</v>
       </c>
@@ -7857,7 +7857,7 @@
       <c r="AH129" s="5"/>
       <c r="AI129" s="5"/>
     </row>
-    <row r="130" spans="1:36" ht="12.75">
+    <row r="130" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A130" s="30" t="s">
         <v>108</v>
       </c>
@@ -7931,15 +7931,15 @@
       </c>
       <c r="S130" s="36">
         <f t="shared" si="9"/>
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="T130" s="36">
         <f t="shared" si="9"/>
-        <v>0.75</v>
+        <v>0.5</v>
       </c>
       <c r="U130" s="36">
         <f t="shared" si="9"/>
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="V130" s="36">
         <f t="shared" si="9"/>
@@ -7980,7 +7980,7 @@
       <c r="AH130" s="5"/>
       <c r="AI130" s="5"/>
     </row>
-    <row r="131" spans="1:36" ht="12.75">
+    <row r="131" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A131" s="30" t="s">
         <v>109</v>
       </c>
@@ -8054,15 +8054,15 @@
       </c>
       <c r="S131" s="36">
         <f t="shared" si="10"/>
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="T131" s="36">
         <f t="shared" si="10"/>
-        <v>0.75</v>
+        <v>0.5</v>
       </c>
       <c r="U131" s="36">
         <f t="shared" si="10"/>
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="V131" s="36">
         <f t="shared" si="10"/>
@@ -8103,7 +8103,7 @@
       <c r="AH131" s="5"/>
       <c r="AI131" s="5"/>
     </row>
-    <row r="132" spans="1:36" ht="12.75">
+    <row r="132" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A132" s="30" t="s">
         <v>110</v>
       </c>
@@ -8173,15 +8173,15 @@
       </c>
       <c r="R132" s="36">
         <f t="shared" si="11"/>
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="S132" s="36">
         <f t="shared" si="11"/>
-        <v>0.75</v>
+        <v>0.5</v>
       </c>
       <c r="T132" s="36">
         <f t="shared" si="11"/>
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="U132" s="36">
         <f t="shared" si="11"/>
@@ -8226,7 +8226,7 @@
       <c r="AH132" s="5"/>
       <c r="AI132" s="5"/>
     </row>
-    <row r="133" spans="1:36" ht="12.75">
+    <row r="133" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A133" s="30" t="s">
         <v>111</v>
       </c>
@@ -8300,15 +8300,15 @@
       </c>
       <c r="S133" s="36">
         <f t="shared" si="12"/>
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="T133" s="36">
         <f t="shared" si="12"/>
-        <v>0.75</v>
+        <v>0.5</v>
       </c>
       <c r="U133" s="36">
         <f t="shared" si="12"/>
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="V133" s="36">
         <f t="shared" si="12"/>
@@ -8349,7 +8349,7 @@
       <c r="AH133" s="5"/>
       <c r="AI133" s="5"/>
     </row>
-    <row r="134" spans="1:36" ht="12.75">
+    <row r="134" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A134" s="30" t="s">
         <v>129</v>
       </c>
@@ -8415,15 +8415,15 @@
       </c>
       <c r="Q134" s="36">
         <f t="shared" si="13"/>
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="R134" s="36">
         <f t="shared" si="13"/>
-        <v>0.75</v>
+        <v>0.5</v>
       </c>
       <c r="S134" s="36">
         <f t="shared" si="13"/>
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="T134" s="36">
         <f t="shared" si="13"/>
@@ -8473,7 +8473,7 @@
       <c r="AI134" s="5"/>
       <c r="AJ134" s="5"/>
     </row>
-    <row r="135" spans="1:36" ht="12.75">
+    <row r="135" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A135" s="13"/>
       <c r="B135" s="5"/>
       <c r="C135" s="5"/>
@@ -8511,7 +8511,7 @@
       <c r="AI135" s="5"/>
       <c r="AJ135" s="5"/>
     </row>
-    <row r="136" spans="1:36" ht="12.75">
+    <row r="136" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A136" s="30" t="s">
         <v>56</v>
       </c>
@@ -8553,7 +8553,7 @@
       <c r="AI136" s="5"/>
       <c r="AJ136" s="5"/>
     </row>
-    <row r="137" spans="1:36" ht="12.75">
+    <row r="137" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A137" s="30" t="s">
         <v>57</v>
       </c>
@@ -8595,7 +8595,7 @@
       <c r="AI137" s="5"/>
       <c r="AJ137" s="5"/>
     </row>
-    <row r="138" spans="1:36" ht="12.75">
+    <row r="138" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A138" s="30" t="s">
         <v>49</v>
       </c>
@@ -8637,7 +8637,7 @@
       <c r="AI138" s="5"/>
       <c r="AJ138" s="5"/>
     </row>
-    <row r="139" spans="1:36" ht="12.75">
+    <row r="139" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A139" s="30" t="s">
         <v>50</v>
       </c>
@@ -8679,7 +8679,7 @@
       <c r="AI139" s="5"/>
       <c r="AJ139" s="5"/>
     </row>
-    <row r="140" spans="1:36" ht="12.75">
+    <row r="140" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A140" s="5" t="s">
         <v>51</v>
       </c>
@@ -8721,7 +8721,7 @@
       <c r="AI140" s="5"/>
       <c r="AJ140" s="5"/>
     </row>
-    <row r="141" spans="1:36" ht="12.75">
+    <row r="141" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A141" s="30" t="s">
         <v>52</v>
       </c>
@@ -8763,7 +8763,7 @@
       <c r="AI141" s="5"/>
       <c r="AJ141" s="5"/>
     </row>
-    <row r="142" spans="1:36" ht="12.75">
+    <row r="142" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A142" s="30" t="s">
         <v>53</v>
       </c>
@@ -8805,7 +8805,7 @@
       <c r="AI142" s="5"/>
       <c r="AJ142" s="5"/>
     </row>
-    <row r="143" spans="1:36" ht="12.75">
+    <row r="143" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A143" s="13"/>
       <c r="B143" s="5"/>
       <c r="C143" s="5"/>
@@ -8843,7 +8843,7 @@
       <c r="AI143" s="5"/>
       <c r="AJ143" s="5"/>
     </row>
-    <row r="144" spans="1:36" ht="12.75">
+    <row r="144" spans="1:36" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A144" s="40" t="s">
         <v>58</v>
       </c>
@@ -8883,7 +8883,7 @@
       <c r="AI144" s="5"/>
       <c r="AJ144" s="5"/>
     </row>
-    <row r="145" spans="1:74" ht="12.75">
+    <row r="145" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A145" s="30"/>
       <c r="B145" s="30">
         <v>2023</v>
@@ -8977,7 +8977,7 @@
       <c r="AI145" s="5"/>
       <c r="AJ145" s="5"/>
     </row>
-    <row r="146" spans="1:74" ht="12.75">
+    <row r="146" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A146" s="5" t="s">
         <v>112</v>
       </c>
@@ -9076,7 +9076,7 @@
       <c r="AI146" s="5"/>
       <c r="AJ146" s="5"/>
     </row>
-    <row r="147" spans="1:74" ht="12.75">
+    <row r="147" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A147" s="30" t="s">
         <v>102</v>
       </c>
@@ -9116,7 +9116,7 @@
       <c r="AI147" s="5"/>
       <c r="AJ147" s="5"/>
     </row>
-    <row r="148" spans="1:74" ht="12.75">
+    <row r="148" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A148" s="30"/>
       <c r="B148" s="37">
         <v>2023</v>
@@ -9210,7 +9210,7 @@
       <c r="AI148" s="5"/>
       <c r="AJ148" s="5"/>
     </row>
-    <row r="149" spans="1:74" ht="12.75">
+    <row r="149" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A149" s="5" t="s">
         <v>113</v>
       </c>
@@ -9284,15 +9284,15 @@
       </c>
       <c r="S149" s="37">
         <f t="shared" si="14"/>
-        <v>0.41625000000000001</v>
+        <v>0.31218750000000001</v>
       </c>
       <c r="T149" s="37">
         <f t="shared" si="14"/>
-        <v>0.31218750000000001</v>
+        <v>0.208125</v>
       </c>
       <c r="U149" s="37">
         <f t="shared" si="14"/>
-        <v>0.208125</v>
+        <v>0</v>
       </c>
       <c r="V149" s="37">
         <f t="shared" si="14"/>
@@ -9334,7 +9334,7 @@
       <c r="AI149" s="5"/>
       <c r="AJ149" s="5"/>
     </row>
-    <row r="150" spans="1:74" ht="12.75">
+    <row r="150" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A150" s="5"/>
       <c r="B150" s="37"/>
       <c r="C150" s="37"/>
@@ -9372,7 +9372,7 @@
       <c r="AI150" s="5"/>
       <c r="AJ150" s="5"/>
     </row>
-    <row r="151" spans="1:74" ht="12.75">
+    <row r="151" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A151" s="30"/>
       <c r="B151" s="37">
         <v>2023</v>
@@ -9466,7 +9466,7 @@
       <c r="AI151" s="5"/>
       <c r="AJ151" s="5"/>
     </row>
-    <row r="152" spans="1:74" ht="12.75">
+    <row r="152" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A152" s="5" t="s">
         <v>114</v>
       </c>
@@ -9536,15 +9536,15 @@
       </c>
       <c r="R152" s="37">
         <f t="shared" si="15"/>
-        <v>0.41625000000000001</v>
+        <v>0.31218750000000001</v>
       </c>
       <c r="S152" s="37">
         <f t="shared" si="15"/>
-        <v>0.31218750000000001</v>
+        <v>0.208125</v>
       </c>
       <c r="T152" s="37">
         <f t="shared" si="15"/>
-        <v>0.208125</v>
+        <v>0</v>
       </c>
       <c r="U152" s="37">
         <f t="shared" si="15"/>
@@ -9590,7 +9590,7 @@
       <c r="AI152" s="5"/>
       <c r="AJ152" s="5"/>
     </row>
-    <row r="153" spans="1:74" ht="12.75">
+    <row r="153" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A153" s="30"/>
       <c r="B153" s="37"/>
       <c r="C153" s="37"/>
@@ -9628,7 +9628,7 @@
       <c r="AI153" s="5"/>
       <c r="AJ153" s="5"/>
     </row>
-    <row r="154" spans="1:74" ht="12.75">
+    <row r="154" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A154" s="30"/>
       <c r="B154" s="37">
         <v>2023</v>
@@ -9722,7 +9722,7 @@
       <c r="AI154" s="5"/>
       <c r="AJ154" s="5"/>
     </row>
-    <row r="155" spans="1:74" ht="12.75">
+    <row r="155" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A155" s="5" t="s">
         <v>59</v>
       </c>
@@ -9796,15 +9796,15 @@
       </c>
       <c r="S155" s="37">
         <f t="shared" si="16"/>
-        <v>0.41625000000000001</v>
+        <v>0.31218750000000001</v>
       </c>
       <c r="T155" s="37">
         <f t="shared" si="16"/>
-        <v>0.31218750000000001</v>
+        <v>0.208125</v>
       </c>
       <c r="U155" s="37">
         <f t="shared" si="16"/>
-        <v>0.208125</v>
+        <v>0</v>
       </c>
       <c r="V155" s="37">
         <f t="shared" si="16"/>
@@ -9846,7 +9846,7 @@
       <c r="AI155" s="5"/>
       <c r="AJ155" s="5"/>
     </row>
-    <row r="156" spans="1:74" ht="12.75">
+    <row r="156" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A156" s="5"/>
       <c r="B156" s="37"/>
       <c r="C156" s="37"/>
@@ -9884,7 +9884,7 @@
       <c r="AI156" s="5"/>
       <c r="AJ156" s="5"/>
     </row>
-    <row r="157" spans="1:74" ht="12.75">
+    <row r="157" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A157" s="30"/>
       <c r="B157" s="37">
         <v>2023</v>
@@ -9978,7 +9978,7 @@
       <c r="AI157" s="5"/>
       <c r="AJ157" s="5"/>
     </row>
-    <row r="158" spans="1:74" ht="12.75">
+    <row r="158" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A158" s="5" t="s">
         <v>127</v>
       </c>
@@ -10044,15 +10044,15 @@
       </c>
       <c r="Q158" s="37">
         <f t="shared" si="17"/>
-        <v>0.41625000000000001</v>
+        <v>0.31218750000000001</v>
       </c>
       <c r="R158" s="37">
         <f t="shared" si="17"/>
-        <v>0.31218750000000001</v>
+        <v>0.208125</v>
       </c>
       <c r="S158" s="37">
         <f t="shared" si="17"/>
-        <v>0.208125</v>
+        <v>0</v>
       </c>
       <c r="T158" s="37">
         <f t="shared" si="17"/>
@@ -10102,7 +10102,7 @@
       <c r="AI158" s="5"/>
       <c r="AJ158" s="5"/>
     </row>
-    <row r="159" spans="1:74" s="35" customFormat="1" ht="12.75">
+    <row r="159" spans="1:74" s="35" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A159" s="32" t="s">
         <v>115</v>
       </c>
@@ -10142,7 +10142,7 @@
       <c r="AI159" s="34"/>
       <c r="AJ159" s="34"/>
     </row>
-    <row r="160" spans="1:74" ht="12.75">
+    <row r="160" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A160" s="5"/>
       <c r="B160" s="5">
         <v>2023</v>
@@ -10274,7 +10274,7 @@
       <c r="BU160" s="5"/>
       <c r="BV160" s="5"/>
     </row>
-    <row r="161" spans="1:74" ht="12.75">
+    <row r="161" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A161" s="5" t="s">
         <v>116</v>
       </c>
@@ -10436,7 +10436,7 @@
       <c r="BU161" s="5"/>
       <c r="BV161" s="5"/>
     </row>
-    <row r="162" spans="1:74" ht="12.75">
+    <row r="162" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A162" s="5" t="s">
         <v>117</v>
       </c>
@@ -10570,7 +10570,7 @@
       <c r="BU162" s="5"/>
       <c r="BV162" s="5"/>
     </row>
-    <row r="163" spans="1:74" ht="12.75">
+    <row r="163" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A163" s="5"/>
       <c r="B163" s="27"/>
       <c r="C163" s="27"/>
@@ -10646,7 +10646,7 @@
       <c r="BU163" s="5"/>
       <c r="BV163" s="5"/>
     </row>
-    <row r="164" spans="1:74" ht="12.75">
+    <row r="164" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A164" s="5" t="s">
         <v>54</v>
       </c>
@@ -10808,7 +10808,7 @@
       <c r="BU164" s="5"/>
       <c r="BV164" s="5"/>
     </row>
-    <row r="165" spans="1:74" ht="12.75">
+    <row r="165" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A165" s="5" t="s">
         <v>93</v>
       </c>
@@ -10874,15 +10874,15 @@
       </c>
       <c r="Q165" s="53">
         <f t="shared" si="19"/>
-        <v>23.051383025144418</v>
+        <v>17.288537268858313</v>
       </c>
       <c r="R165" s="53">
         <f t="shared" si="19"/>
-        <v>17.288537268858313</v>
+        <v>11.525691512572209</v>
       </c>
       <c r="S165" s="53">
         <f t="shared" si="19"/>
-        <v>11.525691512572209</v>
+        <v>0</v>
       </c>
       <c r="T165" s="53">
         <f t="shared" si="19"/>
@@ -10970,7 +10970,7 @@
       <c r="BU165" s="5"/>
       <c r="BV165" s="5"/>
     </row>
-    <row r="166" spans="1:74" ht="12.75">
+    <row r="166" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A166" s="5"/>
       <c r="B166" s="53"/>
       <c r="C166" s="53"/>
@@ -11046,7 +11046,7 @@
       <c r="BU166" s="5"/>
       <c r="BV166" s="5"/>
     </row>
-    <row r="167" spans="1:74" ht="12.75">
+    <row r="167" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A167" s="5" t="s">
         <v>118</v>
       </c>
@@ -11126,7 +11126,7 @@
       <c r="BU167" s="5"/>
       <c r="BV167" s="5"/>
     </row>
-    <row r="168" spans="1:74" ht="12.75">
+    <row r="168" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A168" s="5" t="s">
         <v>119</v>
       </c>
@@ -11288,7 +11288,7 @@
       <c r="BU168" s="5"/>
       <c r="BV168" s="5"/>
     </row>
-    <row r="169" spans="1:74" ht="12.75">
+    <row r="169" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A169" s="5" t="s">
         <v>120</v>
       </c>
@@ -11368,7 +11368,7 @@
       <c r="BU169" s="5"/>
       <c r="BV169" s="5"/>
     </row>
-    <row r="170" spans="1:74" ht="12.75">
+    <row r="170" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A170" s="5" t="s">
         <v>121</v>
       </c>
@@ -11448,7 +11448,7 @@
       <c r="BU170" s="5"/>
       <c r="BV170" s="5"/>
     </row>
-    <row r="171" spans="1:74" ht="12.75">
+    <row r="171" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A171" s="5"/>
       <c r="B171" s="5"/>
       <c r="C171" s="5"/>
@@ -11524,7 +11524,7 @@
       <c r="BU171" s="5"/>
       <c r="BV171" s="5"/>
     </row>
-    <row r="172" spans="1:74" ht="12.75">
+    <row r="172" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A172" s="5" t="s">
         <v>122</v>
       </c>
@@ -11686,7 +11686,7 @@
       <c r="BU172" s="5"/>
       <c r="BV172" s="5"/>
     </row>
-    <row r="173" spans="1:74" ht="12.75">
+    <row r="173" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A173" s="5" t="s">
         <v>123</v>
       </c>
@@ -11752,15 +11752,15 @@
       </c>
       <c r="Q173" s="54">
         <f t="shared" si="22"/>
-        <v>5048252.8825066276</v>
+        <v>3786189.6618799707</v>
       </c>
       <c r="R173" s="54">
         <f t="shared" si="22"/>
-        <v>3786189.6618799707</v>
+        <v>2524126.4412533138</v>
       </c>
       <c r="S173" s="54">
         <f t="shared" si="22"/>
-        <v>2524126.4412533138</v>
+        <v>0</v>
       </c>
       <c r="T173" s="54">
         <f t="shared" si="22"/>
@@ -11848,7 +11848,7 @@
       <c r="BU173" s="5"/>
       <c r="BV173" s="5"/>
     </row>
-    <row r="174" spans="1:74" ht="12.75">
+    <row r="174" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A174" s="5" t="s">
         <v>124</v>
       </c>
@@ -11914,15 +11914,15 @@
       </c>
       <c r="Q174" s="54">
         <f t="shared" si="23"/>
-        <v>47179933.481370352</v>
+        <v>35384950.111027762</v>
       </c>
       <c r="R174" s="54">
         <f t="shared" si="23"/>
-        <v>35384950.111027762</v>
+        <v>23589966.740685176</v>
       </c>
       <c r="S174" s="54">
         <f t="shared" si="23"/>
-        <v>23589966.740685176</v>
+        <v>0</v>
       </c>
       <c r="T174" s="54">
         <f t="shared" si="23"/>
@@ -12010,7 +12010,7 @@
       <c r="BU174" s="5"/>
       <c r="BV174" s="5"/>
     </row>
-    <row r="175" spans="1:74" ht="12.75">
+    <row r="175" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A175" s="5" t="s">
         <v>125</v>
       </c>
@@ -12076,15 +12076,15 @@
       </c>
       <c r="Q175" s="54">
         <f t="shared" si="24"/>
-        <v>50482528.825066276</v>
+        <v>37861896.618799709</v>
       </c>
       <c r="R175" s="54">
         <f t="shared" si="24"/>
-        <v>37861896.618799709</v>
+        <v>25241264.412533138</v>
       </c>
       <c r="S175" s="54">
         <f t="shared" si="24"/>
-        <v>25241264.412533138</v>
+        <v>0</v>
       </c>
       <c r="T175" s="54">
         <f t="shared" si="24"/>
@@ -12172,7 +12172,7 @@
       <c r="BU175" s="5"/>
       <c r="BV175" s="5"/>
     </row>
-    <row r="176" spans="1:74" ht="12.75">
+    <row r="176" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A176" s="5"/>
       <c r="B176" s="5"/>
       <c r="C176" s="5"/>
@@ -12248,7 +12248,7 @@
       <c r="BU176" s="5"/>
       <c r="BV176" s="5"/>
     </row>
-    <row r="177" spans="1:74" ht="12.75">
+    <row r="177" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A177" s="5" t="s">
         <v>126</v>
       </c>
@@ -12410,7 +12410,7 @@
       <c r="BU177" s="5"/>
       <c r="BV177" s="5"/>
     </row>
-    <row r="178" spans="1:74" ht="12.75">
+    <row r="178" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A178" s="5"/>
       <c r="B178" s="5"/>
       <c r="C178" s="5"/>
@@ -12486,7 +12486,7 @@
       <c r="BU178" s="5"/>
       <c r="BV178" s="5"/>
     </row>
-    <row r="179" spans="1:74" ht="12.75">
+    <row r="179" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A179" s="5"/>
       <c r="B179" s="5"/>
       <c r="C179" s="5"/>
@@ -12562,7 +12562,7 @@
       <c r="BU179" s="5"/>
       <c r="BV179" s="5"/>
     </row>
-    <row r="180" spans="1:74" ht="12.75">
+    <row r="180" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A180" s="5"/>
       <c r="B180" s="5"/>
       <c r="C180" s="5"/>
@@ -12638,7 +12638,7 @@
       <c r="BU180" s="5"/>
       <c r="BV180" s="5"/>
     </row>
-    <row r="181" spans="1:74" ht="12.75">
+    <row r="181" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A181" s="5"/>
       <c r="B181" s="5"/>
       <c r="C181" s="5"/>
@@ -12714,7 +12714,7 @@
       <c r="BU181" s="5"/>
       <c r="BV181" s="5"/>
     </row>
-    <row r="182" spans="1:74" ht="12.75">
+    <row r="182" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A182" s="5"/>
       <c r="B182" s="5"/>
       <c r="C182" s="5"/>
@@ -12790,7 +12790,7 @@
       <c r="BU182" s="5"/>
       <c r="BV182" s="5"/>
     </row>
-    <row r="183" spans="1:74" ht="12.75">
+    <row r="183" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A183" s="5"/>
       <c r="B183" s="5"/>
       <c r="C183" s="5"/>
@@ -12866,7 +12866,7 @@
       <c r="BU183" s="5"/>
       <c r="BV183" s="5"/>
     </row>
-    <row r="184" spans="1:74" ht="12.75">
+    <row r="184" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A184" s="5"/>
       <c r="B184" s="5"/>
       <c r="C184" s="5"/>
@@ -12942,7 +12942,7 @@
       <c r="BU184" s="5"/>
       <c r="BV184" s="5"/>
     </row>
-    <row r="185" spans="1:74" ht="12.75">
+    <row r="185" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A185" s="5"/>
       <c r="B185" s="5"/>
       <c r="C185" s="5"/>
@@ -13018,7 +13018,7 @@
       <c r="BU185" s="5"/>
       <c r="BV185" s="5"/>
     </row>
-    <row r="186" spans="1:74" ht="12.75">
+    <row r="186" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A186" s="5"/>
       <c r="B186" s="5"/>
       <c r="C186" s="5"/>
@@ -13094,7 +13094,7 @@
       <c r="BU186" s="5"/>
       <c r="BV186" s="5"/>
     </row>
-    <row r="187" spans="1:74" ht="12.75">
+    <row r="187" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A187" s="5"/>
       <c r="B187" s="5"/>
       <c r="C187" s="5"/>
@@ -13170,7 +13170,7 @@
       <c r="BU187" s="5"/>
       <c r="BV187" s="5"/>
     </row>
-    <row r="188" spans="1:74" ht="12.75">
+    <row r="188" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A188" s="5"/>
       <c r="B188" s="5"/>
       <c r="C188" s="5"/>
@@ -13246,7 +13246,7 @@
       <c r="BU188" s="5"/>
       <c r="BV188" s="5"/>
     </row>
-    <row r="189" spans="1:74" ht="12.75">
+    <row r="189" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A189" s="5"/>
       <c r="B189" s="5"/>
       <c r="C189" s="5"/>
@@ -13322,7 +13322,7 @@
       <c r="BU189" s="5"/>
       <c r="BV189" s="5"/>
     </row>
-    <row r="190" spans="1:74" ht="12.75">
+    <row r="190" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A190" s="5"/>
       <c r="B190" s="5"/>
       <c r="C190" s="5"/>
@@ -13398,7 +13398,7 @@
       <c r="BU190" s="5"/>
       <c r="BV190" s="5"/>
     </row>
-    <row r="191" spans="1:74" ht="12.75">
+    <row r="191" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A191" s="5"/>
       <c r="B191" s="5"/>
       <c r="C191" s="5"/>
@@ -13474,7 +13474,7 @@
       <c r="BU191" s="5"/>
       <c r="BV191" s="5"/>
     </row>
-    <row r="192" spans="1:74" ht="12.75">
+    <row r="192" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A192" s="5"/>
       <c r="B192" s="5"/>
       <c r="C192" s="5"/>
@@ -13550,7 +13550,7 @@
       <c r="BU192" s="5"/>
       <c r="BV192" s="5"/>
     </row>
-    <row r="193" spans="1:74" ht="12.75">
+    <row r="193" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A193" s="5"/>
       <c r="B193" s="5"/>
       <c r="C193" s="5"/>
@@ -13626,7 +13626,7 @@
       <c r="BU193" s="5"/>
       <c r="BV193" s="5"/>
     </row>
-    <row r="194" spans="1:74" ht="12.75">
+    <row r="194" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A194" s="5"/>
       <c r="B194" s="5"/>
       <c r="C194" s="5"/>
@@ -13702,7 +13702,7 @@
       <c r="BU194" s="5"/>
       <c r="BV194" s="5"/>
     </row>
-    <row r="195" spans="1:74" ht="12.75">
+    <row r="195" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A195" s="5"/>
       <c r="B195" s="5"/>
       <c r="C195" s="5"/>
@@ -13778,7 +13778,7 @@
       <c r="BU195" s="5"/>
       <c r="BV195" s="5"/>
     </row>
-    <row r="196" spans="1:74" ht="12.75">
+    <row r="196" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A196" s="5"/>
       <c r="B196" s="5"/>
       <c r="C196" s="5"/>
@@ -13854,7 +13854,7 @@
       <c r="BU196" s="5"/>
       <c r="BV196" s="5"/>
     </row>
-    <row r="197" spans="1:74" ht="12.75">
+    <row r="197" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A197" s="5"/>
       <c r="B197" s="5"/>
       <c r="C197" s="5"/>
@@ -13930,7 +13930,7 @@
       <c r="BU197" s="5"/>
       <c r="BV197" s="5"/>
     </row>
-    <row r="198" spans="1:74" ht="12.75">
+    <row r="198" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A198" s="5"/>
       <c r="B198" s="5"/>
       <c r="C198" s="5"/>
@@ -14006,7 +14006,7 @@
       <c r="BU198" s="5"/>
       <c r="BV198" s="5"/>
     </row>
-    <row r="199" spans="1:74" ht="12.75">
+    <row r="199" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A199" s="5"/>
       <c r="B199" s="5"/>
       <c r="C199" s="5"/>
@@ -14082,7 +14082,7 @@
       <c r="BU199" s="5"/>
       <c r="BV199" s="5"/>
     </row>
-    <row r="200" spans="1:74" ht="12.75">
+    <row r="200" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A200" s="5"/>
       <c r="B200" s="5"/>
       <c r="C200" s="5"/>
@@ -14158,7 +14158,7 @@
       <c r="BU200" s="5"/>
       <c r="BV200" s="5"/>
     </row>
-    <row r="201" spans="1:74" ht="12.75">
+    <row r="201" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A201" s="5"/>
       <c r="B201" s="5"/>
       <c r="C201" s="5"/>
@@ -14234,7 +14234,7 @@
       <c r="BU201" s="5"/>
       <c r="BV201" s="5"/>
     </row>
-    <row r="202" spans="1:74" ht="12.75">
+    <row r="202" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A202" s="5"/>
       <c r="B202" s="5"/>
       <c r="C202" s="5"/>
@@ -14310,7 +14310,7 @@
       <c r="BU202" s="5"/>
       <c r="BV202" s="5"/>
     </row>
-    <row r="203" spans="1:74" ht="12.75">
+    <row r="203" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A203" s="5"/>
       <c r="B203" s="5"/>
       <c r="C203" s="5"/>
@@ -14386,7 +14386,7 @@
       <c r="BU203" s="5"/>
       <c r="BV203" s="5"/>
     </row>
-    <row r="204" spans="1:74" ht="12.75">
+    <row r="204" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A204" s="5"/>
       <c r="B204" s="5"/>
       <c r="C204" s="5"/>
@@ -14462,7 +14462,7 @@
       <c r="BU204" s="5"/>
       <c r="BV204" s="5"/>
     </row>
-    <row r="205" spans="1:74" ht="12.75">
+    <row r="205" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A205" s="5"/>
       <c r="B205" s="5"/>
       <c r="C205" s="5"/>
@@ -14538,7 +14538,7 @@
       <c r="BU205" s="5"/>
       <c r="BV205" s="5"/>
     </row>
-    <row r="206" spans="1:74" ht="12.75">
+    <row r="206" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A206" s="5"/>
       <c r="B206" s="5"/>
       <c r="C206" s="5"/>
@@ -14614,7 +14614,7 @@
       <c r="BU206" s="5"/>
       <c r="BV206" s="5"/>
     </row>
-    <row r="207" spans="1:74" ht="12.75">
+    <row r="207" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A207" s="5"/>
       <c r="B207" s="5"/>
       <c r="C207" s="5"/>
@@ -14690,7 +14690,7 @@
       <c r="BU207" s="5"/>
       <c r="BV207" s="5"/>
     </row>
-    <row r="208" spans="1:74" ht="12.75">
+    <row r="208" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A208" s="5"/>
       <c r="B208" s="5"/>
       <c r="C208" s="5"/>
@@ -14766,7 +14766,7 @@
       <c r="BU208" s="5"/>
       <c r="BV208" s="5"/>
     </row>
-    <row r="209" spans="1:74" ht="12.75">
+    <row r="209" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A209" s="5"/>
       <c r="B209" s="5"/>
       <c r="C209" s="5"/>
@@ -14842,7 +14842,7 @@
       <c r="BU209" s="5"/>
       <c r="BV209" s="5"/>
     </row>
-    <row r="210" spans="1:74" ht="12.75">
+    <row r="210" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A210" s="5"/>
       <c r="B210" s="5"/>
       <c r="C210" s="5"/>
@@ -14918,7 +14918,7 @@
       <c r="BU210" s="5"/>
       <c r="BV210" s="5"/>
     </row>
-    <row r="211" spans="1:74" ht="12.75">
+    <row r="211" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A211" s="5"/>
       <c r="B211" s="5"/>
       <c r="C211" s="5"/>
@@ -14994,7 +14994,7 @@
       <c r="BU211" s="5"/>
       <c r="BV211" s="5"/>
     </row>
-    <row r="212" spans="1:74" ht="12.75">
+    <row r="212" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A212" s="5"/>
       <c r="B212" s="5"/>
       <c r="C212" s="5"/>
@@ -15070,7 +15070,7 @@
       <c r="BU212" s="5"/>
       <c r="BV212" s="5"/>
     </row>
-    <row r="213" spans="1:74" ht="12.75">
+    <row r="213" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A213" s="5"/>
       <c r="B213" s="5"/>
       <c r="C213" s="5"/>
@@ -15146,7 +15146,7 @@
       <c r="BU213" s="5"/>
       <c r="BV213" s="5"/>
     </row>
-    <row r="214" spans="1:74" ht="12.75">
+    <row r="214" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A214" s="5"/>
       <c r="B214" s="5"/>
       <c r="C214" s="5"/>
@@ -15222,7 +15222,7 @@
       <c r="BU214" s="5"/>
       <c r="BV214" s="5"/>
     </row>
-    <row r="215" spans="1:74" ht="12.75">
+    <row r="215" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A215" s="5"/>
       <c r="B215" s="5"/>
       <c r="C215" s="5"/>
@@ -15298,7 +15298,7 @@
       <c r="BU215" s="5"/>
       <c r="BV215" s="5"/>
     </row>
-    <row r="216" spans="1:74" ht="12.75">
+    <row r="216" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A216" s="5"/>
       <c r="B216" s="5"/>
       <c r="C216" s="5"/>
@@ -15374,7 +15374,7 @@
       <c r="BU216" s="5"/>
       <c r="BV216" s="5"/>
     </row>
-    <row r="217" spans="1:74" ht="12.75">
+    <row r="217" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A217" s="5"/>
       <c r="B217" s="5"/>
       <c r="C217" s="5"/>
@@ -15450,7 +15450,7 @@
       <c r="BU217" s="5"/>
       <c r="BV217" s="5"/>
     </row>
-    <row r="218" spans="1:74" ht="12.75">
+    <row r="218" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A218" s="5"/>
       <c r="B218" s="5"/>
       <c r="C218" s="5"/>
@@ -15526,7 +15526,7 @@
       <c r="BU218" s="5"/>
       <c r="BV218" s="5"/>
     </row>
-    <row r="219" spans="1:74" ht="12.75">
+    <row r="219" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A219" s="5"/>
       <c r="B219" s="5"/>
       <c r="C219" s="5"/>
@@ -15602,7 +15602,7 @@
       <c r="BU219" s="5"/>
       <c r="BV219" s="5"/>
     </row>
-    <row r="220" spans="1:74" ht="12.75">
+    <row r="220" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A220" s="5"/>
       <c r="B220" s="5"/>
       <c r="C220" s="5"/>
@@ -15678,7 +15678,7 @@
       <c r="BU220" s="5"/>
       <c r="BV220" s="5"/>
     </row>
-    <row r="221" spans="1:74" ht="12.75">
+    <row r="221" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A221" s="5"/>
       <c r="B221" s="5"/>
       <c r="C221" s="5"/>
@@ -15754,7 +15754,7 @@
       <c r="BU221" s="5"/>
       <c r="BV221" s="5"/>
     </row>
-    <row r="222" spans="1:74" ht="12.75">
+    <row r="222" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A222" s="5"/>
       <c r="B222" s="5"/>
       <c r="C222" s="5"/>
@@ -15830,7 +15830,7 @@
       <c r="BU222" s="5"/>
       <c r="BV222" s="5"/>
     </row>
-    <row r="223" spans="1:74" ht="12.75">
+    <row r="223" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A223" s="5"/>
       <c r="B223" s="5"/>
       <c r="C223" s="5"/>
@@ -15906,7 +15906,7 @@
       <c r="BU223" s="5"/>
       <c r="BV223" s="5"/>
     </row>
-    <row r="224" spans="1:74" ht="12.75">
+    <row r="224" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A224" s="5"/>
       <c r="B224" s="5"/>
       <c r="C224" s="5"/>
@@ -15982,7 +15982,7 @@
       <c r="BU224" s="5"/>
       <c r="BV224" s="5"/>
     </row>
-    <row r="225" spans="1:74" ht="12.75">
+    <row r="225" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A225" s="5"/>
       <c r="B225" s="5"/>
       <c r="C225" s="5"/>
@@ -16058,7 +16058,7 @@
       <c r="BU225" s="5"/>
       <c r="BV225" s="5"/>
     </row>
-    <row r="226" spans="1:74" ht="12.75">
+    <row r="226" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A226" s="5"/>
       <c r="B226" s="5"/>
       <c r="C226" s="5"/>
@@ -16134,7 +16134,7 @@
       <c r="BU226" s="5"/>
       <c r="BV226" s="5"/>
     </row>
-    <row r="227" spans="1:74" ht="12.75">
+    <row r="227" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A227" s="5"/>
       <c r="B227" s="5"/>
       <c r="C227" s="5"/>
@@ -16210,7 +16210,7 @@
       <c r="BU227" s="5"/>
       <c r="BV227" s="5"/>
     </row>
-    <row r="228" spans="1:74" ht="12.75">
+    <row r="228" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A228" s="5"/>
       <c r="B228" s="5"/>
       <c r="C228" s="5"/>
@@ -16286,7 +16286,7 @@
       <c r="BU228" s="5"/>
       <c r="BV228" s="5"/>
     </row>
-    <row r="229" spans="1:74" ht="12.75">
+    <row r="229" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A229" s="5"/>
       <c r="B229" s="5"/>
       <c r="C229" s="5"/>
@@ -16362,7 +16362,7 @@
       <c r="BU229" s="5"/>
       <c r="BV229" s="5"/>
     </row>
-    <row r="230" spans="1:74" ht="12.75">
+    <row r="230" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A230" s="5"/>
       <c r="B230" s="5"/>
       <c r="C230" s="5"/>
@@ -16438,7 +16438,7 @@
       <c r="BU230" s="5"/>
       <c r="BV230" s="5"/>
     </row>
-    <row r="231" spans="1:74" ht="12.75">
+    <row r="231" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A231" s="5"/>
       <c r="B231" s="5"/>
       <c r="C231" s="5"/>
@@ -16514,7 +16514,7 @@
       <c r="BU231" s="5"/>
       <c r="BV231" s="5"/>
     </row>
-    <row r="232" spans="1:74" ht="12.75">
+    <row r="232" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A232" s="5"/>
       <c r="B232" s="5"/>
       <c r="C232" s="5"/>
@@ -16590,7 +16590,7 @@
       <c r="BU232" s="5"/>
       <c r="BV232" s="5"/>
     </row>
-    <row r="233" spans="1:74" ht="12.75">
+    <row r="233" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A233" s="5"/>
       <c r="B233" s="5"/>
       <c r="C233" s="5"/>
@@ -16666,7 +16666,7 @@
       <c r="BU233" s="5"/>
       <c r="BV233" s="5"/>
     </row>
-    <row r="234" spans="1:74" ht="12.75">
+    <row r="234" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A234" s="5"/>
       <c r="B234" s="5"/>
       <c r="C234" s="5"/>
@@ -16742,7 +16742,7 @@
       <c r="BU234" s="5"/>
       <c r="BV234" s="5"/>
     </row>
-    <row r="235" spans="1:74" ht="12.75">
+    <row r="235" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A235" s="5"/>
       <c r="B235" s="5"/>
       <c r="C235" s="5"/>
@@ -16818,7 +16818,7 @@
       <c r="BU235" s="5"/>
       <c r="BV235" s="5"/>
     </row>
-    <row r="236" spans="1:74" ht="12.75">
+    <row r="236" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A236" s="5"/>
       <c r="B236" s="5"/>
       <c r="C236" s="5"/>
@@ -16894,7 +16894,7 @@
       <c r="BU236" s="5"/>
       <c r="BV236" s="5"/>
     </row>
-    <row r="237" spans="1:74" ht="12.75">
+    <row r="237" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A237" s="5"/>
       <c r="B237" s="5"/>
       <c r="C237" s="5"/>
@@ -16970,7 +16970,7 @@
       <c r="BU237" s="5"/>
       <c r="BV237" s="5"/>
     </row>
-    <row r="238" spans="1:74" ht="12.75">
+    <row r="238" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A238" s="5"/>
       <c r="B238" s="5"/>
       <c r="C238" s="5"/>
@@ -17046,7 +17046,7 @@
       <c r="BU238" s="5"/>
       <c r="BV238" s="5"/>
     </row>
-    <row r="239" spans="1:74" ht="12.75">
+    <row r="239" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A239" s="5"/>
       <c r="B239" s="5"/>
       <c r="C239" s="5"/>
@@ -17122,7 +17122,7 @@
       <c r="BU239" s="5"/>
       <c r="BV239" s="5"/>
     </row>
-    <row r="240" spans="1:74" ht="12.75">
+    <row r="240" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A240" s="5"/>
       <c r="B240" s="5"/>
       <c r="C240" s="5"/>
@@ -17198,7 +17198,7 @@
       <c r="BU240" s="5"/>
       <c r="BV240" s="5"/>
     </row>
-    <row r="241" spans="1:74" ht="12.75">
+    <row r="241" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A241" s="5"/>
       <c r="B241" s="5"/>
       <c r="C241" s="5"/>
@@ -17274,7 +17274,7 @@
       <c r="BU241" s="5"/>
       <c r="BV241" s="5"/>
     </row>
-    <row r="242" spans="1:74" ht="12.75">
+    <row r="242" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A242" s="5"/>
       <c r="B242" s="5"/>
       <c r="C242" s="5"/>
@@ -17312,7 +17312,7 @@
       <c r="AI242" s="5"/>
       <c r="AJ242" s="5"/>
     </row>
-    <row r="243" spans="1:74" ht="12.75">
+    <row r="243" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A243" s="5"/>
       <c r="B243" s="5"/>
       <c r="C243" s="5"/>
@@ -17350,7 +17350,7 @@
       <c r="AI243" s="5"/>
       <c r="AJ243" s="5"/>
     </row>
-    <row r="244" spans="1:74" ht="12.75">
+    <row r="244" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A244" s="5"/>
       <c r="B244" s="5"/>
       <c r="C244" s="5"/>
@@ -17388,7 +17388,7 @@
       <c r="AI244" s="5"/>
       <c r="AJ244" s="5"/>
     </row>
-    <row r="245" spans="1:74" ht="12.75">
+    <row r="245" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A245" s="5"/>
       <c r="B245" s="5"/>
       <c r="C245" s="5"/>
@@ -17426,7 +17426,7 @@
       <c r="AI245" s="5"/>
       <c r="AJ245" s="5"/>
     </row>
-    <row r="246" spans="1:74" ht="12.75">
+    <row r="246" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A246" s="5"/>
       <c r="B246" s="5"/>
       <c r="C246" s="5"/>
@@ -17464,7 +17464,7 @@
       <c r="AI246" s="5"/>
       <c r="AJ246" s="5"/>
     </row>
-    <row r="247" spans="1:74" ht="12.75">
+    <row r="247" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A247" s="5"/>
       <c r="B247" s="5"/>
       <c r="C247" s="5"/>
@@ -17502,7 +17502,7 @@
       <c r="AI247" s="5"/>
       <c r="AJ247" s="5"/>
     </row>
-    <row r="248" spans="1:74" ht="12.75">
+    <row r="248" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A248" s="5"/>
       <c r="B248" s="5"/>
       <c r="C248" s="5"/>
@@ -17540,7 +17540,7 @@
       <c r="AI248" s="5"/>
       <c r="AJ248" s="5"/>
     </row>
-    <row r="249" spans="1:74" ht="12.75">
+    <row r="249" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A249" s="5"/>
       <c r="B249" s="5"/>
       <c r="C249" s="5"/>
@@ -17578,7 +17578,7 @@
       <c r="AI249" s="5"/>
       <c r="AJ249" s="5"/>
     </row>
-    <row r="250" spans="1:74" ht="12.75">
+    <row r="250" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A250" s="5"/>
       <c r="B250" s="5"/>
       <c r="C250" s="5"/>
@@ -17616,7 +17616,7 @@
       <c r="AI250" s="5"/>
       <c r="AJ250" s="5"/>
     </row>
-    <row r="251" spans="1:74" ht="12.75">
+    <row r="251" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A251" s="5"/>
       <c r="B251" s="5"/>
       <c r="C251" s="5"/>
@@ -17654,7 +17654,7 @@
       <c r="AI251" s="5"/>
       <c r="AJ251" s="5"/>
     </row>
-    <row r="252" spans="1:74" ht="12.75">
+    <row r="252" spans="1:74" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A252" s="5"/>
       <c r="B252" s="5"/>
       <c r="C252" s="5"/>
@@ -17710,12 +17710,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AE2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -17810,7 +17810,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:31" ht="30">
+    <row r="2" spans="1:31" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>3</v>
       </c>
@@ -17882,15 +17882,15 @@
       </c>
       <c r="S2" s="2">
         <f>'Inflation Reduction Act - Elec'!Q158</f>
-        <v>0.41625000000000001</v>
+        <v>0.31218750000000001</v>
       </c>
       <c r="T2" s="2">
         <f>'Inflation Reduction Act - Elec'!R158</f>
-        <v>0.31218750000000001</v>
+        <v>0.208125</v>
       </c>
       <c r="U2" s="2">
         <f>'Inflation Reduction Act - Elec'!S158</f>
-        <v>0.208125</v>
+        <v>0</v>
       </c>
       <c r="V2" s="2">
         <f>'Inflation Reduction Act - Elec'!T158</f>

</xml_diff>

<commit_message>
Integrate 4.0.4: commit #df12340, 3/11/25, Documentation updates ("latest calibration year target passed" line)
</commit_message>
<xml_diff>
--- a/InputData/elec/BPSpUGBCD/BAU Subsidy per Unit Grid Battery Capacity Deployed.xlsx
+++ b/InputData/elec/BPSpUGBCD/BAU Subsidy per Unit Grid Battery Capacity Deployed.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanO'Brien\Models\EPS\US\eps-us\InputData\elec\BPSpUGBCD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D378A23B-1048-4F0E-9691-78F9E5763631}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06D91A34-2174-4507-BA1E-9A033349103E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1320" yWindow="1200" windowWidth="24750" windowHeight="14490" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1890" yWindow="1200" windowWidth="25275" windowHeight="12525" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>

</xml_diff>